<commit_message>
Release v2.1 SocialPost n8n courseware
</commit_message>
<xml_diff>
--- a/labs/lab-08-multi-channel-content-factory/data/content_matrix.xlsx
+++ b/labs/lab-08-multi-channel-content-factory/data/content_matrix.xlsx
@@ -439,16 +439,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:N5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="17" customWidth="1" min="4" max="4"/>
-    <col width="21" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="19" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="17" customWidth="1" min="11" max="11"/>
+    <col width="21" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -459,30 +466,65 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>brief_id</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>evidence_ids</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>channel</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>format</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>media_type</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>caption</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>media_path</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>user</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>max_chars</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>message_angle</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>cta</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>status</t>
         </is>
@@ -496,28 +538,59 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>BRF-001</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>SRC-001|SRC-002</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
           <t>website</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>landing hero</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>180</v>
-      </c>
       <c r="E2" t="inlineStr">
         <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Audit-ready campaign ROI</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Connect campaign activity to qualified demand</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Book an ROI diagnostic</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>northstar_training</t>
+        </is>
+      </c>
+      <c r="K2" t="n">
+        <v>1800</v>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
           <t>audit-ready ROI</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="M2" t="inlineStr">
         <is>
           <t>Book diagnostic</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t>draft</t>
         </is>
@@ -531,28 +604,59 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
+          <t>BRF-001</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>SRC-001|SRC-002</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
           <t>linkedin</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>single post</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Prove campaign contribution</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Evidence-led benchmark for SG marketing teams</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Read the benchmark</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>northstar_training</t>
+        </is>
+      </c>
+      <c r="K3" t="n">
         <v>1300</v>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t>prove contribution</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="M3" t="inlineStr">
         <is>
           <t>Read benchmark</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="N3" t="inlineStr">
         <is>
           <t>draft</t>
         </is>
@@ -566,28 +670,133 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>email</t>
+          <t>BRF-001</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>nurture email</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>1800</v>
+          <t>SRC-001|SRC-002</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>instagram</t>
+        </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>reduce reporting friction</t>
+          <t>photos</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Book diagnostic</t>
+          <t>Northstar campaign evidence</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
+        <is>
+          <t>A visual summary of auditable campaign decisions</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Review the evidence</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>media/northstar-carousel-01.png</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>northstar_training</t>
+        </is>
+      </c>
+      <c r="K4" t="n">
+        <v>2200</v>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>show evidence</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Review evidence</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>AST-004</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>BRF-001</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>SRC-001|SRC-002</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>youtube</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Northstar evidence briefing</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>A short evidence-led campaign briefing</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Watch the evidence briefing</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>media/northstar-evidence-video.mp4</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>northstar_training</t>
+        </is>
+      </c>
+      <c r="K5" t="n">
+        <v>5000</v>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>explain the evidence</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Watch briefing</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
         <is>
           <t>draft</t>
         </is>
@@ -604,7 +813,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -649,7 +858,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>channel</t>
+          <t>brief_id</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -659,14 +868,14 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>website</t>
+          <t>BRF-001</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>format</t>
+          <t>evidence_ids</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -676,14 +885,14 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>landing hero</t>
+          <t>SRC-001|SRC-002</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>max_chars</t>
+          <t>channel</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -691,14 +900,16 @@
           <t>Input/output field used by Lab 8</t>
         </is>
       </c>
-      <c r="C5" t="n">
-        <v>180</v>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>website</t>
+        </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>message_angle</t>
+          <t>media_type</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -708,14 +919,14 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>audit-ready ROI</t>
+          <t>text</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>cta</t>
+          <t>title</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -725,22 +936,135 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Book diagnostic</t>
+          <t>Audit-ready campaign ROI</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Input/output field used by Lab 8</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Connect campaign activity to qualified demand</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>caption</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Input/output field used by Lab 8</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Book an ROI diagnostic</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>media_path</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Input/output field used by Lab 8</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>user</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Input/output field used by Lab 8</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>northstar_training</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>max_chars</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Input/output field used by Lab 8</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>1800</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>message_angle</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Input/output field used by Lab 8</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>audit-ready ROI</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>cta</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Input/output field used by Lab 8</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Book diagnostic</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
           <t>status</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Input/output field used by Lab 8</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Input/output field used by Lab 8</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
         <is>
           <t>draft</t>
         </is>
@@ -780,7 +1104,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Acceptance check: One approved brief produces distinct channel assets; every asset retains brief_id, evidence_ids and validation status.</t>
+          <t>Acceptance check: One approved brief produces distinct channel assets; every social asset is endpoint-ready and retains brief_id, evidence_ids and validation status.</t>
         </is>
       </c>
     </row>

</xml_diff>